<commit_message>
chore: refresh HIRA material outputs
</commit_message>
<xml_diff>
--- a/hira_material_automation/output/monthly/202601_202607__acl_interference_screw_absorbable__040012__normalized.xlsx
+++ b/hira_material_automation/output/monthly/202601_202607__acl_interference_screw_absorbable__040012__normalized.xlsx
@@ -711,7 +711,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-04T22:02:50</t>
+          <t>2026-07-14T22:02:40</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>84718659bda8653634ce3c143350c309154825a084f7aa358e5b504ed6a798af</t>
+          <t>e3e9436e1f7f450189eac4d28621aef86f06f12642063030f6b4a0cb71cb1970</t>
         </is>
       </c>
     </row>

</xml_diff>